<commit_message>
feat: adiciona o log no git
</commit_message>
<xml_diff>
--- a/log/log_execucoes.xlsx
+++ b/log/log_execucoes.xlsx
@@ -80,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -114,6 +114,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -483,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -569,49 +572,49 @@
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>EXE_20260323_095800</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>23/03/2026 09:58:00</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>23/03/2026 11:07:55</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>1h 09m 54s</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F2" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="9" t="n">
+      <c r="F2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="9" t="n">
+      <c r="I2" s="12" t="n">
         <v>405</v>
       </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -621,52 +624,52 @@
           <t>✅ benchmarkComposicaoDeCustos</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr"/>
+      <c r="M2" s="12" t="inlineStr"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>EXE_20260323_112655</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>23/03/2026 11:26:55</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>23/03/2026 14:01:28</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>2h 34m 32s</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F3" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="9" t="n">
+      <c r="F3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="9" t="n">
+      <c r="I3" s="12" t="n">
         <v>3637</v>
       </c>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="K3" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -676,52 +679,52 @@
           <t>✅ benchmarkComposicaoDeCustos</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr"/>
+      <c r="M3" s="12" t="inlineStr"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>EXE_20260323_144448</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>23/03/2026 14:44:48</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>23/03/2026 15:57:12</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>1h 12m 23s</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="9" t="n">
+      <c r="F4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="9" t="n">
+      <c r="I4" s="12" t="n">
         <v>3637</v>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -731,52 +734,52 @@
           <t>✅ benchmarkComposicaoDeCustos</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr"/>
+      <c r="M4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>EXE_20260324_152806</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>24/03/2026 15:28:06</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>24/03/2026 18:01:25</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>2h 33m 19s</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F5" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="9" t="n">
+      <c r="F5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="12" t="n">
         <v>13373</v>
       </c>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -786,52 +789,52 @@
           <t>✅ demonstracaoCustoUnitarioDosServicosAuxiliares</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr"/>
+      <c r="M5" s="12" t="inlineStr"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>EXE_20260330_095828</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>30/03/2026 09:58:28</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>30/03/2026 13:01:46</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>3h 03m 17s</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="9" t="n">
+      <c r="F6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="12" t="n">
         <v>13396</v>
       </c>
-      <c r="J6" s="9" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -841,52 +844,52 @@
           <t>✅ demonstracaoCustoUnitarioDosServicosAuxiliares</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr"/>
+      <c r="M6" s="12" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>EXE_20260330_133153</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>30/03/2026 13:31:53</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>30/03/2026 15:50:19</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>2h 18m 25s</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F7" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="9" t="n">
+      <c r="F7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="12" t="n">
         <v>13396</v>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="K7" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -896,52 +899,52 @@
           <t>✅ demonstracaoCustoUnitarioDosServicosAuxiliares</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr"/>
+      <c r="M7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>EXE_20260331_093010</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>31/03/2026 09:30:10</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>31/03/2026 12:05:47</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>2h 35m 37s</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\02_2026</t>
         </is>
       </c>
-      <c r="F8" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="9" t="n">
+      <c r="F8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I8" s="12" t="n">
         <v>13367</v>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>processar</t>
         </is>
       </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="K8" s="12" t="inlineStr">
         <is>
           <t>Sucesso Total</t>
         </is>
@@ -951,7 +954,7 @@
           <t>✅ demonstracaoCustoUnitarioDosServicosAuxiliares</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr"/>
+      <c r="M8" s="12" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -1062,6 +1065,61 @@
         </is>
       </c>
       <c r="M10" s="12" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>EXE_20260505_144402</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>05/05/2026 14:44:02</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>05/05/2026 16:05:43</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>1h 21m 41s</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Y:\CONTROLADORIA\CUSTOS\16_BASES_KPIH\2026\04_2026</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>128927</v>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>processar</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>Sucesso Total</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>✅ Consumo | ✅ QuantidadeLeito | ✅ QuantidadeCirurgia | ✅ NotasFiscais | ✅ FolhadePagamento | ✅ custosIndividualizadoPorCentro | ✅ producoes | ✅ estatistica | ✅ rankingDeCusto | ✅ evolucaoDeCustos | ✅ demonstracaoCustoUnitario | ✅ demonstracaoCustoUnitarioPorSaida | ✅ painelComparativoDeCustos | ✅ custoPorEspecialidade | ✅ analisedepartamental | ✅ composicaoDeCustos | ✅ composicaoEvolucaoDeReceita | ✅ custoUnitarioPorPonderacao | ✅ demonstracaoCustoUnitarioDosServicosAuxiliares | ✅ benchmarkComposicaoDeCustos</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>